<commit_message>
Record ASTRA shared runtime mission execution
</commit_message>
<xml_diff>
--- a/canonical/astra_runtime/tmp/XLSX_LIBRARY_ROUNDTRIP_VERIFY.xlsx
+++ b/canonical/astra_runtime/tmp/XLSX_LIBRARY_ROUNDTRIP_VERIFY.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
   <si>
     <t>capability_id</t>
   </si>
@@ -116,6 +116,18 @@
   </si>
   <si>
     <t>["python.tests.audit"]</t>
+  </si>
+  <si>
+    <t>xlsx.table.create_from_json_records</t>
+  </si>
+  <si>
+    <t>["xlsx.table.create_from_json_records"]</t>
+  </si>
+  <si>
+    <t>xlsx.table.verify_against_json_records</t>
+  </si>
+  <si>
+    <t>["xlsx.table.verify_against_json_records"]</t>
   </si>
   <si>
     <t>yaml.to_json.yq</t>
@@ -453,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -694,6 +706,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>